<commit_message>
feat: added symmetrical pitch, gavel sound, and manual timer logic
</commit_message>
<xml_diff>
--- a/match_roster.xlsx
+++ b/match_roster.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AYAN\auction-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8DAE7CB-2E67-4E58-ABBA-127CA4808DA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0495B7CB-17B7-4957-833C-792F299C65D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9C81F2A8-E914-47DA-B05A-D76E35A54E9A}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="74">
   <si>
     <t>Name</t>
   </si>
@@ -181,16 +181,97 @@
   </si>
   <si>
     <t>Dhwanit</t>
+  </si>
+  <si>
+    <t>8 goals</t>
+  </si>
+  <si>
+    <t>9 goals</t>
+  </si>
+  <si>
+    <t>10 goals</t>
+  </si>
+  <si>
+    <t>11 goals</t>
+  </si>
+  <si>
+    <t>12 goals</t>
+  </si>
+  <si>
+    <t>13 goals</t>
+  </si>
+  <si>
+    <t>14 goals</t>
+  </si>
+  <si>
+    <t>15 goals</t>
+  </si>
+  <si>
+    <t>16 goals</t>
+  </si>
+  <si>
+    <t>17 goals</t>
+  </si>
+  <si>
+    <t>18 goals</t>
+  </si>
+  <si>
+    <t>19 goals</t>
+  </si>
+  <si>
+    <t>20 goals</t>
+  </si>
+  <si>
+    <t>21 goals</t>
+  </si>
+  <si>
+    <t>22 goals</t>
+  </si>
+  <si>
+    <t>23 goals</t>
+  </si>
+  <si>
+    <t>24 goals</t>
+  </si>
+  <si>
+    <t>25 goals</t>
+  </si>
+  <si>
+    <t>26 goals</t>
+  </si>
+  <si>
+    <t>27 goals</t>
+  </si>
+  <si>
+    <t>28 goals</t>
+  </si>
+  <si>
+    <t>29 goals</t>
+  </si>
+  <si>
+    <t>30 goals</t>
+  </si>
+  <si>
+    <t>31 goals</t>
+  </si>
+  <si>
+    <t>Last Match Stats</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -553,7 +634,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BA29EC4-0059-495C-A18E-E59E0D501DA6}">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.88671875" bestFit="1" customWidth="1"/>
@@ -563,7 +644,7 @@
     <col min="5" max="5" width="14.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -579,8 +660,11 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -596,8 +680,11 @@
       <c r="E2" s="1">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F2" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
@@ -613,8 +700,11 @@
       <c r="E3" s="1">
         <v>6.5</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F3" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -630,8 +720,11 @@
       <c r="E4" s="1">
         <v>8.5</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F4" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
@@ -647,8 +740,11 @@
       <c r="E5" s="1">
         <v>7.5</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F5" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
@@ -664,8 +760,11 @@
       <c r="E6" s="1">
         <v>6.5</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F6" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
@@ -681,8 +780,11 @@
       <c r="E7" s="1">
         <v>7.5</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F7" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -698,8 +800,11 @@
       <c r="E8" s="1">
         <v>7.5</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F8" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>22</v>
       </c>
@@ -715,8 +820,11 @@
       <c r="E9" s="1">
         <v>5</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F9" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>23</v>
       </c>
@@ -732,8 +840,11 @@
       <c r="E10" s="1">
         <v>5.5</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F10" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>24</v>
       </c>
@@ -749,8 +860,11 @@
       <c r="E11" s="1">
         <v>8</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F11" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>26</v>
       </c>
@@ -766,8 +880,11 @@
       <c r="E12" s="1">
         <v>7.5</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F12" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>28</v>
       </c>
@@ -783,8 +900,11 @@
       <c r="E13" s="1">
         <v>6.5</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F13" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>29</v>
       </c>
@@ -800,8 +920,11 @@
       <c r="E14" s="1">
         <v>7</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F14" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>31</v>
       </c>
@@ -817,8 +940,11 @@
       <c r="E15" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F15" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>33</v>
       </c>
@@ -834,8 +960,11 @@
       <c r="E16" s="1">
         <v>6</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F16" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>35</v>
       </c>
@@ -851,8 +980,11 @@
       <c r="E17" s="1">
         <v>7</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F17" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>36</v>
       </c>
@@ -868,8 +1000,11 @@
       <c r="E18" s="1">
         <v>7</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F18" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>38</v>
       </c>
@@ -885,8 +1020,11 @@
       <c r="E19" s="1">
         <v>5.5</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F19" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>40</v>
       </c>
@@ -902,8 +1040,11 @@
       <c r="E20" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F20" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>42</v>
       </c>
@@ -919,8 +1060,11 @@
       <c r="E21" s="1">
         <v>7.5</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F21" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>43</v>
       </c>
@@ -936,8 +1080,11 @@
       <c r="E22" s="1">
         <v>5.5</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F22" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>45</v>
       </c>
@@ -953,8 +1100,11 @@
       <c r="E23" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F23" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>47</v>
       </c>
@@ -970,8 +1120,11 @@
       <c r="E24" s="1">
         <v>5</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F24" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>48</v>
       </c>
@@ -987,8 +1140,12 @@
       <c r="E25" s="1">
         <v>5.5</v>
       </c>
+      <c r="F25" s="1" t="s">
+        <v>72</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>